<commit_message>
Update government grants: 2027 3억, 2028+ 1억/yr
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T42GPG2qKtV2XApvVvEGav
</commit_message>
<xml_diff>
--- a/모닛_5개년_사업계획_손익계산서_2026-2030.xlsx
+++ b/모닛_5개년_사업계획_손익계산서_2026-2030.xlsx
@@ -1747,23 +1747,23 @@
       </c>
       <c r="E14" s="17">
         <f>'3_연간손익'!E21/100000</f>
-        <v>5.201748408</v>
+        <v>7.801748408</v>
       </c>
       <c r="F14" s="17">
         <f>'3_연간손익'!F21/100000</f>
-        <v>31.215806495802</v>
+        <v>31.189806495802</v>
       </c>
       <c r="G14" s="17">
         <f>'3_연간손익'!G21/100000</f>
-        <v>70.3705552468748</v>
+        <v>71.1505552468748</v>
       </c>
       <c r="H14" s="17">
         <f>'3_연간손익'!H21/100000</f>
-        <v>190.436387193969</v>
+        <v>191.194387193969</v>
       </c>
       <c r="I14" s="14">
         <f>IFERROR(('3_연간손익'!H21/'3_연간손익'!C21)^(1/5)-1,"n/a")</f>
-        <v>4.16772250041508</v>
+        <v>4.17182981621665</v>
       </c>
     </row>
     <row r="15">
@@ -9042,71 +9042,71 @@
       </c>
       <c r="P46" s="25">
         <f>P47</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="Q46" s="25">
         <f>Q47</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="R46" s="25">
         <f>R47</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="S46" s="25">
         <f>S47</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="T46" s="25">
         <f>T47</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="U46" s="25">
         <f>U47</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="V46" s="25">
         <f>V47</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="W46" s="25">
         <f>W47</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="X46" s="25">
         <f>X47</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="Y46" s="25">
         <f>Y47</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="Z46" s="25">
         <f>Z47</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="AA46" s="25">
         <f>AA47</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="AB46" s="23">
         <f>AB47</f>
-        <v>40000</v>
+        <v>300000</v>
       </c>
       <c r="AC46" s="34">
         <f>AC47</f>
-        <v>30000</v>
+        <v>100000</v>
       </c>
       <c r="AD46" s="34">
         <f>AD47</f>
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="AE46" s="34">
         <f>AE47</f>
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="AF46" s="25">
         <f>AF47</f>
-        <v>365000</v>
+        <v>895000</v>
       </c>
     </row>
     <row r="47">
@@ -9169,71 +9169,71 @@
       </c>
       <c r="P47" s="40">
         <f>'7_비용인력'!P33</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="Q47" s="40">
         <f>'7_비용인력'!Q33</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="R47" s="40">
         <f>'7_비용인력'!R33</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="S47" s="40">
         <f>'7_비용인력'!S33</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="T47" s="40">
         <f>'7_비용인력'!T33</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="U47" s="40">
         <f>'7_비용인력'!U33</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="V47" s="40">
         <f>'7_비용인력'!V33</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="W47" s="40">
         <f>'7_비용인력'!W33</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="X47" s="40">
         <f>'7_비용인력'!X33</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="Y47" s="40">
         <f>'7_비용인력'!Y33</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="Z47" s="40">
         <f>'7_비용인력'!Z33</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="AA47" s="40">
         <f>'7_비용인력'!AA33</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="AB47" s="41">
         <f>'7_비용인력'!AB33</f>
-        <v>40000</v>
+        <v>300000</v>
       </c>
       <c r="AC47" s="42">
         <f>'7_비용인력'!AC33</f>
-        <v>30000</v>
+        <v>100000</v>
       </c>
       <c r="AD47" s="42">
         <f>'7_비용인력'!AD33</f>
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="AE47" s="42">
         <f>'7_비용인력'!AE33</f>
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="AF47" s="40">
         <f>'7_비용인력'!AF33</f>
-        <v>365000</v>
+        <v>895000</v>
       </c>
     </row>
     <row r="48">
@@ -9550,71 +9550,71 @@
       </c>
       <c r="P50" s="26">
         <f>P42+P46-P48</f>
-        <v>-61943.7656112995</v>
+        <v>-40277.0989446328</v>
       </c>
       <c r="Q50" s="26">
         <f>Q42+Q46-Q48</f>
-        <v>-40101.7930390163</v>
+        <v>-18435.1263723496</v>
       </c>
       <c r="R50" s="26">
         <f>R42+R46-R48</f>
-        <v>-18259.8204667332</v>
+        <v>3406.8461999335</v>
       </c>
       <c r="S50" s="26">
         <f>S42+S46-S48</f>
-        <v>3164.1860038551</v>
+        <v>24830.8526705218</v>
       </c>
       <c r="T50" s="26">
         <f>T42+T46-T48</f>
-        <v>24588.1924744433</v>
+        <v>46254.85914111</v>
       </c>
       <c r="U50" s="26">
         <f>U42+U46-U48</f>
-        <v>64462.1989450316</v>
+        <v>86128.8656116983</v>
       </c>
       <c r="V50" s="26">
         <f>V42+V46-V48</f>
-        <v>84132.6054156198</v>
+        <v>105799.272082286</v>
       </c>
       <c r="W50" s="26">
         <f>W42+W46-W48</f>
-        <v>101279.83541562</v>
+        <v>122946.502082287</v>
       </c>
       <c r="X50" s="26">
         <f>X42+X46-X48</f>
-        <v>99977.0654156198</v>
+        <v>121643.732082287</v>
       </c>
       <c r="Y50" s="26">
         <f>Y42+Y46-Y48</f>
-        <v>94683.4854156198</v>
+        <v>116350.152082286</v>
       </c>
       <c r="Z50" s="26">
         <f>Z42+Z46-Z48</f>
-        <v>89389.9054156198</v>
+        <v>111056.572082286</v>
       </c>
       <c r="AA50" s="26">
         <f>AA42+AA46-AA48</f>
-        <v>78802.7454156198</v>
+        <v>100469.412082287</v>
       </c>
       <c r="AB50" s="27">
         <f>AB42+AB46-AB48</f>
-        <v>520174.8408</v>
+        <v>780174.8408</v>
       </c>
       <c r="AC50" s="28">
         <f>AC42+AC46-AC48</f>
-        <v>3251540.94148028</v>
+        <v>3321540.94148028</v>
       </c>
       <c r="AD50" s="28">
         <f>AD42+AD46-AD48</f>
-        <v>8993660.92908651</v>
+        <v>9093660.92908651</v>
       </c>
       <c r="AE50" s="28">
         <f>AE42+AE46-AE48</f>
-        <v>24514035.249864</v>
+        <v>24614035.249864</v>
       </c>
       <c r="AF50" s="26">
         <f>AF42+AF46-AF48</f>
-        <v>37230506.7784964</v>
+        <v>37760506.7784964</v>
       </c>
     </row>
     <row r="51">
@@ -9734,19 +9734,19 @@
       </c>
       <c r="AC51" s="24">
         <f>'7_비용인력'!AC49</f>
-        <v>129960.291900081</v>
+        <v>202560.291900081</v>
       </c>
       <c r="AD51" s="24">
         <f>'7_비용인력'!AD49</f>
-        <v>1956605.40439903</v>
+        <v>1978605.40439903</v>
       </c>
       <c r="AE51" s="24">
         <f>'7_비용인력'!AE49</f>
-        <v>5470396.53046709</v>
+        <v>5494596.53046709</v>
       </c>
       <c r="AF51" s="25">
         <f>O51+AB51+AC51+AD51+AE51</f>
-        <v>7556962.2267662</v>
+        <v>7675762.2267662</v>
       </c>
     </row>
     <row r="52">
@@ -9809,71 +9809,71 @@
       </c>
       <c r="P52" s="37">
         <f>P50-P51</f>
-        <v>-61943.7656112995</v>
+        <v>-40277.0989446328</v>
       </c>
       <c r="Q52" s="37">
         <f>Q50-Q51</f>
-        <v>-40101.7930390163</v>
+        <v>-18435.1263723496</v>
       </c>
       <c r="R52" s="37">
         <f>R50-R51</f>
-        <v>-18259.8204667332</v>
+        <v>3406.8461999335</v>
       </c>
       <c r="S52" s="37">
         <f>S50-S51</f>
-        <v>3164.1860038551</v>
+        <v>24830.8526705218</v>
       </c>
       <c r="T52" s="37">
         <f>T50-T51</f>
-        <v>24588.1924744433</v>
+        <v>46254.85914111</v>
       </c>
       <c r="U52" s="37">
         <f>U50-U51</f>
-        <v>64462.1989450316</v>
+        <v>86128.8656116983</v>
       </c>
       <c r="V52" s="37">
         <f>V50-V51</f>
-        <v>84132.6054156198</v>
+        <v>105799.272082286</v>
       </c>
       <c r="W52" s="37">
         <f>W50-W51</f>
-        <v>101279.83541562</v>
+        <v>122946.502082287</v>
       </c>
       <c r="X52" s="37">
         <f>X50-X51</f>
-        <v>99977.0654156198</v>
+        <v>121643.732082287</v>
       </c>
       <c r="Y52" s="37">
         <f>Y50-Y51</f>
-        <v>94683.4854156198</v>
+        <v>116350.152082286</v>
       </c>
       <c r="Z52" s="37">
         <f>Z50-Z51</f>
-        <v>89389.9054156198</v>
+        <v>111056.572082286</v>
       </c>
       <c r="AA52" s="37">
         <f>AA50-AA51</f>
-        <v>78802.7454156198</v>
+        <v>100469.412082287</v>
       </c>
       <c r="AB52" s="38">
         <f>AB50-AB51</f>
-        <v>520174.8408</v>
+        <v>780174.8408</v>
       </c>
       <c r="AC52" s="39">
         <f>AC50-AC51</f>
-        <v>3121580.6495802</v>
+        <v>3118980.6495802</v>
       </c>
       <c r="AD52" s="39">
         <f>AD50-AD51</f>
-        <v>7037055.52468748</v>
+        <v>7115055.52468748</v>
       </c>
       <c r="AE52" s="39">
         <f>AE50-AE51</f>
-        <v>19043638.7193969</v>
+        <v>19119438.7193969</v>
       </c>
       <c r="AF52" s="37">
         <f>AF50-AF51</f>
-        <v>29673544.5517302</v>
+        <v>30084744.5517302</v>
       </c>
     </row>
     <row r="53">
@@ -9936,71 +9936,71 @@
       </c>
       <c r="P53" s="14">
         <f>IFERROR(P52/P14,0)</f>
-        <v>-0.216581938062771</v>
+        <v>-0.140825990523626</v>
       </c>
       <c r="Q53" s="14">
         <f>IFERROR(Q52/Q14,0)</f>
-        <v>-0.101026354131045</v>
+        <v>-0.0464426516672594</v>
       </c>
       <c r="R53" s="14">
         <f>IFERROR(R52/R14,0)</f>
-        <v>-0.0359529070644745</v>
+        <v>0.00670795340142141</v>
       </c>
       <c r="S53" s="14">
         <f>IFERROR(S52/S14,0)</f>
-        <v>0.00512730632385453</v>
+        <v>0.0402363792043676</v>
       </c>
       <c r="T53" s="14">
         <f>IFERROR(T52/T14,0)</f>
-        <v>0.0338509100725547</v>
+        <v>0.0636797145146736</v>
       </c>
       <c r="U53" s="14">
         <f>IFERROR(U52/U14,0)</f>
-        <v>0.0719757416749849</v>
+        <v>0.0961678174725823</v>
       </c>
       <c r="V53" s="14">
         <f>IFERROR(V52/V14,0)</f>
-        <v>0.0843230257120453</v>
+        <v>0.106038731310394</v>
       </c>
       <c r="W53" s="14">
         <f>IFERROR(W52/W14,0)</f>
-        <v>0.0929615157154855</v>
+        <v>0.112848654804624</v>
       </c>
       <c r="X53" s="14">
         <f>IFERROR(X52/X14,0)</f>
-        <v>0.0891680377393997</v>
+        <v>0.108492211168464</v>
       </c>
       <c r="Y53" s="14">
         <f>IFERROR(Y52/Y14,0)</f>
-        <v>0.0844467735249093</v>
+        <v>0.103770946953973</v>
       </c>
       <c r="Z53" s="14">
         <f>IFERROR(Z52/Z14,0)</f>
-        <v>0.0797255093104189</v>
+        <v>0.099049682739483</v>
       </c>
       <c r="AA53" s="14">
         <f>IFERROR(AA52/AA14,0)</f>
-        <v>0.0702829808814381</v>
+        <v>0.0896071543105022</v>
       </c>
       <c r="AB53" s="30">
         <f>IFERROR(AB52/AB14,0)</f>
-        <v>0.0520068746775658</v>
+        <v>0.0780015717593611</v>
       </c>
       <c r="AC53" s="31">
         <f>IFERROR(AC52/AC14,0)</f>
-        <v>0.0945933530175819</v>
+        <v>0.0945145651387941</v>
       </c>
       <c r="AD53" s="31">
         <f>IFERROR(AD52/AD14,0)</f>
-        <v>0.100529364638393</v>
+        <v>0.101643650352678</v>
       </c>
       <c r="AE53" s="31">
         <f>IFERROR(AE52/AE14,0)</f>
-        <v>0.122074607175621</v>
+        <v>0.122560504611519</v>
       </c>
       <c r="AF53" s="14">
         <f>IFERROR(AF52/AF14,0)</f>
-        <v>0.109819839079417</v>
+        <v>0.111341663266977</v>
       </c>
     </row>
     <row r="54"/>
@@ -11071,19 +11071,19 @@
       </c>
       <c r="E15" s="18">
         <f>'2_손익계산서'!AB46</f>
-        <v>40000</v>
+        <v>300000</v>
       </c>
       <c r="F15" s="18">
         <f>'2_손익계산서'!AC46</f>
-        <v>30000</v>
+        <v>100000</v>
       </c>
       <c r="G15" s="18">
         <f>'2_손익계산서'!AD46</f>
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="H15" s="18">
         <f>'2_손익계산서'!AE46</f>
-        <v>0</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="16">
@@ -11104,19 +11104,19 @@
       </c>
       <c r="E16" s="40">
         <f>'2_손익계산서'!AB47</f>
-        <v>40000</v>
+        <v>300000</v>
       </c>
       <c r="F16" s="40">
         <f>'2_손익계산서'!AC47</f>
-        <v>30000</v>
+        <v>100000</v>
       </c>
       <c r="G16" s="40">
         <f>'2_손익계산서'!AD47</f>
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="H16" s="40">
         <f>'2_손익계산서'!AE47</f>
-        <v>0</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="17">
@@ -11205,19 +11205,19 @@
       </c>
       <c r="E19" s="25">
         <f>E13+E15-E17</f>
-        <v>520174.8408</v>
+        <v>780174.8408</v>
       </c>
       <c r="F19" s="25">
         <f>F13+F15-F17</f>
-        <v>3251540.94148028</v>
+        <v>3321540.94148028</v>
       </c>
       <c r="G19" s="25">
         <f>G13+G15-G17</f>
-        <v>8993660.92908651</v>
+        <v>9093660.92908651</v>
       </c>
       <c r="H19" s="25">
         <f>H13+H15-H17</f>
-        <v>24514035.249864</v>
+        <v>24614035.249864</v>
       </c>
     </row>
     <row r="20">
@@ -11242,15 +11242,15 @@
       </c>
       <c r="F20" s="18">
         <f>'2_손익계산서'!AC51</f>
-        <v>129960.291900081</v>
+        <v>202560.291900081</v>
       </c>
       <c r="G20" s="18">
         <f>'2_손익계산서'!AD51</f>
-        <v>1956605.40439903</v>
+        <v>1978605.40439903</v>
       </c>
       <c r="H20" s="18">
         <f>'2_손익계산서'!AE51</f>
-        <v>5470396.53046709</v>
+        <v>5494596.53046709</v>
       </c>
     </row>
     <row r="21">
@@ -11273,23 +11273,23 @@
       </c>
       <c r="E21" s="37">
         <f>E19-E20</f>
-        <v>520174.8408</v>
+        <v>780174.8408</v>
       </c>
       <c r="F21" s="37">
         <f>F19-F20</f>
-        <v>3121580.6495802</v>
+        <v>3118980.6495802</v>
       </c>
       <c r="G21" s="37">
         <f>G19-G20</f>
-        <v>7037055.52468748</v>
+        <v>7115055.52468748</v>
       </c>
       <c r="H21" s="37">
         <f>H19-H20</f>
-        <v>19043638.7193969</v>
+        <v>19119438.7193969</v>
       </c>
       <c r="I21" s="14">
         <f>IFERROR((H21/C21)^(1/5)-1,"n/a")</f>
-        <v>4.16772250041508</v>
+        <v>4.17182981621665</v>
       </c>
     </row>
     <row r="22">
@@ -11312,19 +11312,19 @@
       </c>
       <c r="E22" s="14">
         <f>IFERROR(E21/E7,0)</f>
-        <v>0.0520068746775658</v>
+        <v>0.0780015717593611</v>
       </c>
       <c r="F22" s="14">
         <f>IFERROR(F21/F7,0)</f>
-        <v>0.0945933530175819</v>
+        <v>0.0945145651387941</v>
       </c>
       <c r="G22" s="14">
         <f>IFERROR(G21/G7,0)</f>
-        <v>0.100529364638393</v>
+        <v>0.101643650352678</v>
       </c>
       <c r="H22" s="14">
         <f>IFERROR(H21/H7,0)</f>
-        <v>0.122074607175621</v>
+        <v>0.122560504611519</v>
       </c>
     </row>
     <row r="23">
@@ -33758,71 +33758,71 @@
       </c>
       <c r="P33" s="18">
         <f>'8_가정'!$D$112/12</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="Q33" s="18">
         <f>'8_가정'!$D$112/12</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="R33" s="18">
         <f>'8_가정'!$D$112/12</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="S33" s="18">
         <f>'8_가정'!$D$112/12</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="T33" s="18">
         <f>'8_가정'!$D$112/12</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="U33" s="18">
         <f>'8_가정'!$D$112/12</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="V33" s="18">
         <f>'8_가정'!$D$112/12</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="W33" s="18">
         <f>'8_가정'!$D$112/12</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="X33" s="18">
         <f>'8_가정'!$D$112/12</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="Y33" s="18">
         <f>'8_가정'!$D$112/12</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="Z33" s="18">
         <f>'8_가정'!$D$112/12</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="AA33" s="18">
         <f>'8_가정'!$D$112/12</f>
-        <v>3333.33333333333</v>
+        <v>25000</v>
       </c>
       <c r="AB33" s="23">
         <f>SUM(P33:AA33)</f>
-        <v>40000</v>
+        <v>300000</v>
       </c>
       <c r="AC33" s="24">
         <f>'8_가정'!$E$112</f>
-        <v>30000</v>
+        <v>100000</v>
       </c>
       <c r="AD33" s="24">
         <f>'8_가정'!$F$112</f>
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="AE33" s="24">
         <f>'8_가정'!$G$112</f>
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="AF33" s="25">
         <f>O33+AB33+AC33+AD33+AE33</f>
-        <v>365000</v>
+        <v>895000</v>
       </c>
     </row>
     <row r="34">
@@ -34059,19 +34059,19 @@
       </c>
       <c r="AB40" s="48">
         <f>'2_손익계산서'!AB50</f>
-        <v>520174.8408</v>
+        <v>780174.8408</v>
       </c>
       <c r="AC40" s="24">
         <f>'2_손익계산서'!AC50</f>
-        <v>3251540.94148028</v>
+        <v>3321540.94148028</v>
       </c>
       <c r="AD40" s="24">
         <f>'2_손익계산서'!AD50</f>
-        <v>8993660.92908651</v>
+        <v>9093660.92908651</v>
       </c>
       <c r="AE40" s="24">
         <f>'2_손익계산서'!AE50</f>
-        <v>24514035.249864</v>
+        <v>24614035.249864</v>
       </c>
     </row>
     <row r="41">
@@ -34090,7 +34090,7 @@
       </c>
       <c r="AC41" s="45">
         <f>AB44</f>
-        <v>2560812.34193446</v>
+        <v>2300812.34193446</v>
       </c>
       <c r="AD41" s="45">
         <f>AC44</f>
@@ -34113,11 +34113,11 @@
       </c>
       <c r="AB42" s="48">
         <f>MIN(AB41,MAX(0,AB40)*'8_가정'!$C$117)</f>
-        <v>520174.8408</v>
+        <v>780174.8408</v>
       </c>
       <c r="AC42" s="24">
         <f>MIN(AC41,MAX(0,AC40)*'8_가정'!$C$117)</f>
-        <v>2560812.34193446</v>
+        <v>2300812.34193446</v>
       </c>
       <c r="AD42" s="24">
         <f>MIN(AD41,MAX(0,AD40)*'8_가정'!$C$117)</f>
@@ -34167,7 +34167,7 @@
       </c>
       <c r="AB44" s="44">
         <f>AB41-AB42+AB43</f>
-        <v>2560812.34193446</v>
+        <v>2300812.34193446</v>
       </c>
       <c r="AC44" s="45">
         <f>AC41-AC42+AC43</f>
@@ -34198,15 +34198,15 @@
       </c>
       <c r="AC45" s="45">
         <f>MAX(0,AC40)-AC42</f>
-        <v>690728.599545821</v>
+        <v>1020728.59954582</v>
       </c>
       <c r="AD45" s="45">
         <f>MAX(0,AD40)-AD42</f>
-        <v>8993660.92908651</v>
+        <v>9093660.92908651</v>
       </c>
       <c r="AE45" s="45">
         <f>MAX(0,AE40)-AE42</f>
-        <v>24514035.249864</v>
+        <v>24614035.249864</v>
       </c>
     </row>
     <row r="46">
@@ -34225,15 +34225,15 @@
       </c>
       <c r="AC46" s="24">
         <f>MIN(AC45,'8_가정'!$C$118)*'8_가정'!$C$119+MAX(0,MIN(AC45,'8_가정'!$D$118)-'8_가정'!$C$118)*'8_가정'!$D$119+MAX(0,MIN(AC45,'8_가정'!$E$118)-'8_가정'!$D$118)*'8_가정'!$E$119+MAX(0,AC45-'8_가정'!$E$118)*'8_가정'!$F$119</f>
-        <v>118145.719909164</v>
+        <v>184145.719909164</v>
       </c>
       <c r="AD46" s="24">
         <f>MIN(AD45,'8_가정'!$C$118)*'8_가정'!$C$119+MAX(0,MIN(AD45,'8_가정'!$D$118)-'8_가정'!$C$118)*'8_가정'!$D$119+MAX(0,MIN(AD45,'8_가정'!$E$118)-'8_가정'!$D$118)*'8_가정'!$E$119+MAX(0,AD45-'8_가정'!$E$118)*'8_가정'!$F$119</f>
-        <v>1778732.1858173</v>
+        <v>1798732.1858173</v>
       </c>
       <c r="AE46" s="24">
         <f>MIN(AE45,'8_가정'!$C$118)*'8_가정'!$C$119+MAX(0,MIN(AE45,'8_가정'!$D$118)-'8_가정'!$C$118)*'8_가정'!$D$119+MAX(0,MIN(AE45,'8_가정'!$E$118)-'8_가정'!$D$118)*'8_가정'!$E$119+MAX(0,AE45-'8_가정'!$E$118)*'8_가정'!$F$119</f>
-        <v>4973087.75497008</v>
+        <v>4995087.75497008</v>
       </c>
     </row>
     <row r="47">
@@ -34252,15 +34252,15 @@
       </c>
       <c r="AC47" s="24">
         <f>AC46*'8_가정'!$C$120</f>
-        <v>11814.5719909164</v>
+        <v>18414.5719909164</v>
       </c>
       <c r="AD47" s="24">
         <f>AD46*'8_가정'!$C$120</f>
-        <v>177873.21858173</v>
+        <v>179873.21858173</v>
       </c>
       <c r="AE47" s="24">
         <f>AE46*'8_가정'!$C$120</f>
-        <v>497308.775497008</v>
+        <v>499508.775497008</v>
       </c>
     </row>
     <row r="48">
@@ -34279,15 +34279,15 @@
       </c>
       <c r="AC48" s="34">
         <f>AC46+AC47</f>
-        <v>129960.291900081</v>
+        <v>202560.291900081</v>
       </c>
       <c r="AD48" s="34">
         <f>AD46+AD47</f>
-        <v>1956605.40439903</v>
+        <v>1978605.40439903</v>
       </c>
       <c r="AE48" s="34">
         <f>AE46+AE47</f>
-        <v>5470396.53046709</v>
+        <v>5494596.53046709</v>
       </c>
     </row>
     <row r="49">
@@ -34402,19 +34402,19 @@
       </c>
       <c r="AC49" s="45">
         <f>AC48</f>
-        <v>129960.291900081</v>
+        <v>202560.291900081</v>
       </c>
       <c r="AD49" s="45">
         <f>AD48</f>
-        <v>1956605.40439903</v>
+        <v>1978605.40439903</v>
       </c>
       <c r="AE49" s="45">
         <f>AE48</f>
-        <v>5470396.53046709</v>
+        <v>5494596.53046709</v>
       </c>
       <c r="AF49" s="25">
         <f>O49+AB49+AC49+AD49+AE49</f>
-        <v>7556962.2267662</v>
+        <v>7675762.2267662</v>
       </c>
     </row>
     <row r="51">
@@ -37220,7 +37220,7 @@
       </c>
       <c r="B112" s="15" t="inlineStr">
         <is>
-          <t>2027~ 입력(보수적 체감)</t>
+          <t>2027: 3억 예상, 2028~: 매년 1억(보수적)</t>
         </is>
       </c>
       <c r="C112" s="96">
@@ -37228,20 +37228,20 @@
         <v>295000</v>
       </c>
       <c r="D112" s="65" t="n">
-        <v>40000</v>
+        <v>300000</v>
       </c>
       <c r="E112" s="65" t="n">
-        <v>30000</v>
+        <v>100000</v>
       </c>
       <c r="F112" s="65" t="n">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="G112" s="65" t="n">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="I112" s="89" t="inlineStr">
         <is>
-          <t>2024 0.88억, 2025 0.31억 실적(영업외수익 처리 선례). 2029~ 미반영</t>
+          <t>2024 0.88억, 2025 0.31억 실적(영업외수익 처리 선례). 2027 3억(사용자 제공), 2028~ 연 1억 보수적 가정(과제 수행 비용 대응 한도 내 확인 필요)</t>
         </is>
       </c>
     </row>
@@ -37673,16 +37673,16 @@
         <v>-0.489051827344633</v>
       </c>
       <c r="D10" s="98" t="n">
-        <v>5.201748408</v>
+        <v>7.801748408</v>
       </c>
       <c r="E10" s="98" t="n">
-        <v>31.215806495802</v>
+        <v>31.189806495802</v>
       </c>
       <c r="F10" s="98" t="n">
-        <v>70.3705552468748</v>
+        <v>71.1505552468748</v>
       </c>
       <c r="G10" s="98" t="n">
-        <v>190.436387193969</v>
+        <v>191.194387193969</v>
       </c>
     </row>
     <row r="11">
@@ -37868,16 +37868,16 @@
         <v>-0.7085080836531791</v>
       </c>
       <c r="D21" s="98" t="n">
-        <v>-2.85410320759547</v>
+        <v>-0.254103207595469</v>
       </c>
       <c r="E21" s="98" t="n">
-        <v>9.378050222007131</v>
+        <v>10.0780502220071</v>
       </c>
       <c r="F21" s="98" t="n">
-        <v>17.8398139060112</v>
+        <v>18.8398139060112</v>
       </c>
       <c r="G21" s="98" t="n">
-        <v>38.4212438145785</v>
+        <v>38.2552438145785</v>
       </c>
     </row>
     <row r="22">
@@ -38063,16 +38063,16 @@
         <v>-1.10018038900559</v>
       </c>
       <c r="D32" s="98" t="n">
-        <v>-6.61343250407795</v>
+        <v>-4.01343250407795</v>
       </c>
       <c r="E32" s="98" t="n">
-        <v>-2.91351714627082</v>
+        <v>-2.21351714627082</v>
       </c>
       <c r="F32" s="98" t="n">
-        <v>-13.572215931278</v>
+        <v>-12.572215931278</v>
       </c>
       <c r="G32" s="98" t="n">
-        <v>-24.2095182039728</v>
+        <v>-23.2095182039728</v>
       </c>
     </row>
     <row r="33">
@@ -38291,19 +38291,19 @@
       </c>
       <c r="D43" s="17">
         <f>'3_연간손익'!E21/100000</f>
-        <v>5.201748408</v>
+        <v>7.801748408</v>
       </c>
       <c r="E43" s="17">
         <f>'3_연간손익'!F21/100000</f>
-        <v>31.215806495802</v>
+        <v>31.189806495802</v>
       </c>
       <c r="F43" s="17">
         <f>'3_연간손익'!G21/100000</f>
-        <v>70.3705552468748</v>
+        <v>71.1505552468748</v>
       </c>
       <c r="G43" s="17">
         <f>'3_연간손익'!H21/100000</f>
-        <v>190.436387193969</v>
+        <v>191.194387193969</v>
       </c>
     </row>
     <row r="44">

</xml_diff>